<commit_message>
Propostas: FOXTERMO (Humberto na equipe + horas) e registro Petrobras
FOXTERMO (Alvaro):
- FOXTERMO_Proposta.xlsx: adiciona coluna Humberto na aba Cronograma,
  reajusta horas do Gabriel (173->105h dividido com Humberto 68h),
  corrige formulas (O4=SUM(K24:M24), % por pessoa). Total R$31.571,43.
- cronograma_horas.md: detalhe das horas por atividade (Marcus/Gabriel/Humberto).

Petrobras (Rui):
- proposta_resumo.md: registro so de fatos (escopo, cronograma, entregaveis)
  + revisao passada ao Marcus. Sem dados bancarios/CNPJ nem valor comercial.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0144GG7dJhKbZ5sWAH3QTbQX
</commit_message>
<xml_diff>
--- a/foxtermo_cristalizacao/FOXTERMO_Proposta.xlsx
+++ b/foxtermo_cristalizacao/FOXTERMO_Proposta.xlsx
@@ -753,7 +753,7 @@
     <xf numFmtId="9" fontId="2" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="23" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="143">
+  <cellXfs count="144">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="8" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -1111,6 +1111,7 @@
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="2"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="10"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="11">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2323,7 +2324,11 @@
           <t>Gabriel</t>
         </is>
       </c>
-      <c r="M3" s="45" t="n"/>
+      <c r="M3" s="46" t="inlineStr">
+        <is>
+          <t>Humberto</t>
+        </is>
+      </c>
       <c r="N3" s="46" t="inlineStr">
         <is>
           <t>Urgência</t>
@@ -2363,7 +2368,7 @@
         </is>
       </c>
       <c r="O4" s="138">
-        <f>SUM(K24:L24)</f>
+        <f>SUM(K24:M24)</f>
         <v/>
       </c>
       <c r="P4" s="50" t="n"/>
@@ -2472,7 +2477,10 @@
         <v>6</v>
       </c>
       <c r="L9" t="n">
-        <v>50</v>
+        <v>30</v>
+      </c>
+      <c r="M9" t="n">
+        <v>20</v>
       </c>
       <c r="N9" s="141" t="n"/>
     </row>
@@ -2521,7 +2529,10 @@
         <v>8</v>
       </c>
       <c r="L13" t="n">
-        <v>70</v>
+        <v>40</v>
+      </c>
+      <c r="M13" t="n">
+        <v>30</v>
       </c>
     </row>
     <row r="14" ht="15" customHeight="1">
@@ -2569,7 +2580,10 @@
         <v>6</v>
       </c>
       <c r="L17" t="n">
-        <v>45</v>
+        <v>30</v>
+      </c>
+      <c r="M17" t="n">
+        <v>15</v>
       </c>
     </row>
     <row r="18" ht="15" customHeight="1">
@@ -2617,7 +2631,10 @@
         <v>4</v>
       </c>
       <c r="L21" t="n">
-        <v>8</v>
+        <v>5</v>
+      </c>
+      <c r="M21" t="n">
+        <v>3</v>
       </c>
     </row>
     <row r="22">
@@ -2638,6 +2655,10 @@
         <f>SUM(L4:L21)</f>
         <v/>
       </c>
+      <c r="M22">
+        <f>SUM(M4:M21)</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
       <c r="J23" s="46" t="inlineStr">
@@ -2651,6 +2672,10 @@
       </c>
       <c r="L23" s="141">
         <f>VLOOKUP(L3,'Tabela HH'!$H$4:$K$19,IF($O$3="Sim",4,3),0)</f>
+        <v/>
+      </c>
+      <c r="M23" s="138">
+        <f>VLOOKUP(M3,'Tabela HH'!$H$4:$K$19,IF($O$3="Sim",4,3),0)</f>
         <v/>
       </c>
     </row>
@@ -2663,6 +2688,10 @@
         <f>L22*VLOOKUP(L3,'Tabela HH'!$H$4:$K$19,IF($O$3="Sim",4,3),0)</f>
         <v/>
       </c>
+      <c r="M24" s="138">
+        <f>M22*VLOOKUP(M3,'Tabela HH'!$H$4:$K$19,IF($O$3="Sim",4,3),0)</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
       <c r="J25" s="46" t="inlineStr">
@@ -2678,8 +2707,12 @@
         <f>L24/$O$4*$O$6</f>
         <v/>
       </c>
-      <c r="M25" s="74">
-        <f>SUM(K25:L25)</f>
+      <c r="M25" s="143">
+        <f>M24/$O$4*$O$6</f>
+        <v/>
+      </c>
+      <c r="N25" s="143">
+        <f>SUM(K25:M25)</f>
         <v/>
       </c>
     </row>

</xml_diff>